<commit_message>
Fill HSK1_parts_of_speech files 8, 9, 10 (ID 351-500) with parts of speech
</commit_message>
<xml_diff>
--- a/HSK1_parts_of_speech_8(351-400).xlsx
+++ b/HSK1_parts_of_speech_8(351-400).xlsx
@@ -601,6 +601,11 @@
           <t>четыре</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>четыре</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -627,6 +632,11 @@
           <t>отправлять, дарить</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>отправлять, провожать; дарить</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -653,6 +663,16 @@
           <t>год, возраст</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>возраст; год (жизни)</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>для возраста и годов (五岁 — 5 лет)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -679,6 +699,11 @@
           <t>он</t>
         </is>
       </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>он</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -705,6 +730,11 @@
           <t>они</t>
         </is>
       </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>они (мужчины или смешанная группа)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -731,6 +761,11 @@
           <t>она</t>
         </is>
       </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>она</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -757,6 +792,11 @@
           <t>они (о женщинах)</t>
         </is>
       </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>они (о женщинах)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -783,6 +823,11 @@
           <t>слишком</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>слишком; очень (太好了!)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -809,6 +854,11 @@
           <t>день</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>день; небо</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -835,6 +885,16 @@
           <t>погода</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>погода</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>словосочетание (天+气), цельная лексема</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -861,6 +921,11 @@
           <t>слышать</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>слушать, слышать</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -887,6 +952,16 @@
           <t>услышать, дослушать до...</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>услышать, дослушать до...</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>глагол + результативное дополнение</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -913,6 +988,16 @@
           <t>слышать, услышать</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>слышать, услышать</t>
+        </is>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>глагол + результативное дополнение</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -939,6 +1024,21 @@
           <t>диктант</t>
         </is>
       </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>диктант</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>писать под диктовку</t>
+        </is>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>离合词: 听写汉字</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -965,6 +1065,11 @@
           <t>одноклассник</t>
         </is>
       </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>одноклассник; товарищ по учёбе</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -991,6 +1096,11 @@
           <t>библиотека</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>библиотека</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1017,6 +1127,16 @@
           <t>вне</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>наружная сторона, вне (方位词)</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>иностранный, внешний (外国)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1043,6 +1163,11 @@
           <t>снаружи, внешняя сторона</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>снаружи, внешняя сторона (方位词)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1069,6 +1194,16 @@
           <t>иностранное государство</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>иностранное государство</t>
+        </is>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>словосочетание (外+国)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1095,6 +1230,16 @@
           <t>иностранный язык</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>иностранный язык</t>
+        </is>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>словосочетание (外+语)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1121,6 +1266,11 @@
           <t>играть, гулять</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>играть, развлекаться, гулять</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1147,6 +1297,21 @@
           <t>вечер, поздний</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>вечер (今晚)</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>поздний (晚到)</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>поздно</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1173,6 +1338,16 @@
           <t>ужин</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ужин</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>словосочетание (晚+饭)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1199,6 +1374,11 @@
           <t>вечер</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>вечер, nighttime (方位词)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1225,6 +1405,11 @@
           <t>онлайн</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>в интернете, онлайн (方位词)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1251,6 +1436,16 @@
           <t>интернет-друг</t>
         </is>
       </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>интернет-друг, сетевой знакомый</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>словосочетание (网+友)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1277,6 +1472,11 @@
           <t>забывать</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>забывать</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1303,6 +1503,16 @@
           <t>забыть</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>забыть</t>
+        </is>
+      </c>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>глагол + дополнительное значение (忘+记)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1329,6 +1539,11 @@
           <t>спросить</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>спрашивать, задавать вопрос</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1355,6 +1570,11 @@
           <t>я</t>
         </is>
       </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>я</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1381,6 +1601,11 @@
           <t>мы</t>
         </is>
       </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>мы</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1407,6 +1632,11 @@
           <t>пять</t>
         </is>
       </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>пять</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1433,6 +1663,16 @@
           <t>обед</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>обед (полуденная трапеза)</t>
+        </is>
+      </c>
+      <c r="X34" t="inlineStr">
+        <is>
+          <t>словосочетание (午+饭)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1459,6 +1699,11 @@
           <t>запад</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>запад (сторона света)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1485,6 +1730,11 @@
           <t>запад, западная сторона</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>запад, западная сторона (方位词)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1511,6 +1761,11 @@
           <t>мыть</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>мыть, стирать (衣服)、洗手</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1537,6 +1792,16 @@
           <t>уборная</t>
         </is>
       </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>уборная, раковина (место для мытья)</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>словосочетание (洗手间)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1563,6 +1828,11 @@
           <t>любить, нравиться</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>любить, нравиться</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1589,6 +1859,26 @@
           <t>внизу; спускаться</t>
         </is>
       </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>низ (方位词)</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>спускаться; оканчиваться (下车、下课)</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>нижний; следующий (下次)</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>для занятий/раундов (一下、三下)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1615,6 +1905,16 @@
           <t>уходить с работы</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>уходить с работы</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>离合词: 下了班</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1641,6 +1941,11 @@
           <t>под, снизу</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>под, снизу (方位词)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1667,6 +1972,16 @@
           <t>выйти из (машины), сойти с (поезда)</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>выйти из машины, сойти с поезда</t>
+        </is>
+      </c>
+      <c r="X43" t="inlineStr">
+        <is>
+          <t>离合词: 下了车</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1693,6 +2008,16 @@
           <t>следующий раз</t>
         </is>
       </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>следующий раз</t>
+        </is>
+      </c>
+      <c r="X44" t="inlineStr">
+        <is>
+          <t>словосочетание (下+次)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1719,6 +2044,16 @@
           <t>уйти по окончании урока</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>заканчивать урок</t>
+        </is>
+      </c>
+      <c r="X45" t="inlineStr">
+        <is>
+          <t>离合词: 下了课</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1745,6 +2080,11 @@
           <t>после полудня</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>после полудня, вторая половина дня (方位词)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1771,6 +2111,16 @@
           <t>идёт дождь</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>идёт дождь, дождит</t>
+        </is>
+      </c>
+      <c r="X47" t="inlineStr">
+        <is>
+          <t>离合词: 下了一场雨</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1797,6 +2147,16 @@
           <t>сначала</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>очередь (我先)</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>сначала, сперва</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1823,6 +2183,11 @@
           <t>господин</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>господин, мистер; учитель</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1849,6 +2214,16 @@
           <t>сейчас</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>сейчас (时+间 сокращ.)</t>
+        </is>
+      </c>
+      <c r="X50" t="inlineStr">
+        <is>
+          <t>цельная лексема «сейчас»</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1873,6 +2248,11 @@
       <c r="I51" t="inlineStr">
         <is>
           <t>думать, хотеть, скучать</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>думать; хотеть; скучать</t>
         </is>
       </c>
     </row>

</xml_diff>